<commit_message>
Remove six weaker tools (75 tools now) and update maps, paths, templates and preview image
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dXhz1wBJHDaaJTjaDP8MA
</commit_message>
<xml_diff>
--- a/templates/innovation-calculators.xlsx
+++ b/templates/innovation-calculators.xlsx
@@ -11,9 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riskiest Assumption" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup Metrics" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sizing the Raise" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investor Readiness" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spending Gates" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pivot Triggers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spending Gates" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pivot Triggers" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -101,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -118,7 +117,6 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,7 +480,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -595,7 +593,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -603,7 +600,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -782,7 +779,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -790,7 +786,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1039,7 +1035,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1047,7 +1042,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1175,7 +1170,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1183,196 +1177,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:C20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Investor Readiness</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Yellow cells are inputs. Blue cells calculate. Replace the example numbers with your own.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Score each area out of 10. Anything below 5 needs fixing before you pitch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Area</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Score (0-10)</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>What would raise it</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Value proposition</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" s="10" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>Market</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" s="10" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Go-to-market</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C9" s="10" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C10" s="10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C11" s="10" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C12" s="10" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Risks</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C13" s="10" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Milestones</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C14" s="10" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Exit</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C15" s="10" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Lowest score</t>
-        </is>
-      </c>
-      <c r="B17" s="16">
-        <f>MIN(B7:B15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Investor's biggest objection (one sentence)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Your answer (two sentences)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Ready to pitch? Yes, or fix the lowest score first</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1473,15 +1278,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1548,6 +1352,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix logic slips, glossary gaps, spelling and carry-over issues from full read-through
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dXhz1wBJHDaaJTjaDP8MA
</commit_message>
<xml_diff>
--- a/templates/innovation-calculators.xlsx
+++ b/templates/innovation-calculators.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Sizing" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riskiest Assumption" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup Metrics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start-up Metrics" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sizing the Raise" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spending Gates" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pivot Triggers" sheetId="6" state="visible" r:id="rId6"/>
@@ -799,7 +799,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Startup Metrics</t>
+          <t>Start-up Metrics</t>
         </is>
       </c>
     </row>

</xml_diff>